<commit_message>
Beslut om korten: korten gäller först; faskortens B/S/K, kulturkostnad och namn bekräftade
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JCFLjpHxkTTwZndbAW5eBH
</commit_message>
<xml_diff>
--- a/kortdata/GF_faskort.xlsx
+++ b/kortdata/GF_faskort.xlsx
@@ -6565,7 +6565,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B14"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -6731,10 +6731,46 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
+          <t>B/S/K</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Bostad / Special / Komplex — tidigare indelning, samma logik (bekräftat av användaren).</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Kulturkostnad</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Steg 1 = 2 Mkr, steg 2–8 = stegnumret. Avsiktligt: 'andra chans' till samma kostnad när man förstått logiken (bekräftat av användaren).</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Namn</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>De fulla namnen i kolumnen Namn är de rätta; 'Namn som tryckt' visar tryckets avkortning.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
           <t>Byggd med</t>
         </is>
       </c>
-      <c r="B14" s="2" t="inlineStr">
+      <c r="B17" s="2" t="inlineStr">
         <is>
           <t>verktyg/bygg_gf_faskort_excel.py</t>
         </is>

</xml_diff>